<commit_message>
Add Missing photos tab to the master sheet.
42 SKUs have no picture (blank swatch on the site). Custom 99999999
is not a hide. Photograph or pull art for the rest.
</commit_message>
<xml_diff>
--- a/docs/Furniture Information Sheet.xlsx
+++ b/docs/Furniture Information Sheet.xlsx
@@ -8,16 +8,18 @@
   </bookViews>
   <sheets>
     <sheet name="To complete" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Catalog" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Medium — confirm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="New — need SKUs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Price differences" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Missing photos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Catalog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Medium — confirm" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="New — need SKUs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Price differences" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalog'!$A$1:$V$200</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Medium — confirm'!$A$1:$G$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'New — need SKUs'!$A$1:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price differences'!$A$1:$G$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Missing photos'!$A$1:$I$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Catalog'!$A$1:$V$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Medium — confirm'!$A$1:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'New — need SKUs'!$A$1:$H$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Price differences'!$A$1:$G$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,6 +55,10 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00F4EFE6"/>
     </font>
   </fonts>
   <fills count="7">
@@ -114,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -142,6 +148,8 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -529,6 +537,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -682,6 +691,24 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>9. Photograph or pull art for Missing photos tab</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Missing photos tab</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>42 SKUs have no picture — blank swatch on the site</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
@@ -710,6 +737,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
@@ -720,6 +748,1381 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>sku</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>hide</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>on_hand</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>ss_item</t>
+        </is>
+      </c>
+      <c r="H1" s="14" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="I1" s="14" t="inlineStr">
+        <is>
+          <t>why</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>50701239</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>Antoinette</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>White Croc Front, Cowhide Back</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="n">
+        <v>1699</v>
+      </c>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="13" t="n"/>
+      <c r="G2" s="13" t="n"/>
+      <c r="H2" s="13" t="n"/>
+      <c r="I2" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>50701843</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Antoinette</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>All brown leather</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="n">
+        <v>1699</v>
+      </c>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="13" t="n"/>
+      <c r="G3" s="13" t="n"/>
+      <c r="H3" s="13" t="n"/>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>50701833</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Antoinette</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Brindle Front Brown Croc Back</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="n">
+        <v>1699</v>
+      </c>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="13" t="n"/>
+      <c r="G4" s="13" t="n"/>
+      <c r="H4" s="13" t="n"/>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>50701002</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Antoinette</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Brown Croc Front</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>1699</v>
+      </c>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="13" t="n"/>
+      <c r="G5" s="13" t="n"/>
+      <c r="H5" s="13" t="n"/>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>50701202</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Antoinette</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Brown croc Front black, white hide Back</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>1699</v>
+      </c>
+      <c r="E6" s="13" t="n"/>
+      <c r="F6" s="13" t="n"/>
+      <c r="G6" s="13" t="n"/>
+      <c r="H6" s="13" t="n"/>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>50701834</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Antoinette</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Dark Brindle Front Brown Croc Back</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>1699</v>
+      </c>
+      <c r="E7" s="13" t="n"/>
+      <c r="F7" s="13" t="n"/>
+      <c r="G7" s="13" t="n"/>
+      <c r="H7" s="13" t="n"/>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>50701832</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Antoinette</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>white Brindle Front Brown Croc Back</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>1699</v>
+      </c>
+      <c r="E8" s="13" t="n"/>
+      <c r="F8" s="13" t="n"/>
+      <c r="G8" s="13" t="n"/>
+      <c r="H8" s="13" t="n"/>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>30310223</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Bethany</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Top Brown Croc back OLD</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>650</v>
+      </c>
+      <c r="E9" s="13" t="n"/>
+      <c r="F9" s="13" t="n"/>
+      <c r="G9" s="13" t="n"/>
+      <c r="H9" s="13" t="n"/>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>11111</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Brooke</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>600</v>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>Brooke Brown Barstool</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>Placeholder SKU Brooke Brown Barstool | 600 on master vs 400 at Sunset Sage</t>
+        </is>
+      </c>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>55304124</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Fufu</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Ivory</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>200</v>
+      </c>
+      <c r="E11" s="13" t="n"/>
+      <c r="F11" s="13" t="n"/>
+      <c r="G11" s="13" t="n"/>
+      <c r="H11" s="13" t="n"/>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>30268454</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>George</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Legs Short Brown</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>350</v>
+      </c>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="13" t="n"/>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>30268545</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>George</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Legs Tall Brown</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="n">
+        <v>350</v>
+      </c>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+      <c r="H13" s="13" t="n"/>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>30268843</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>George</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Top Grey Leather</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>350</v>
+      </c>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="13" t="n"/>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>11307002</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Grace</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>Dark Croc</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>650</v>
+      </c>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="13" t="n"/>
+      <c r="G15" s="13" t="n"/>
+      <c r="H15" s="13" t="n"/>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>11307003</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Grace</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>White Croc</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>650</v>
+      </c>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="13" t="n"/>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Levi</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="E17" s="13" t="n"/>
+      <c r="F17" s="13" t="n"/>
+      <c r="G17" s="13" t="n"/>
+      <c r="H17" s="13" t="n"/>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Levi</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="13" t="n"/>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Levi</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>Taupe</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>30180124</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Lincoln</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>Light brown &amp; Hide trim</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="13" t="n"/>
+      <c r="G20" s="13" t="n"/>
+      <c r="H20" s="13" t="n"/>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>30216193</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Marlo</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>Old All grey leather</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="n">
+        <v>350</v>
+      </c>
+      <c r="E21" s="13" t="n"/>
+      <c r="F21" s="13" t="n"/>
+      <c r="G21" s="13" t="n"/>
+      <c r="H21" s="13" t="n"/>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>30216172</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Marlo</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>Old Brown croc</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="n">
+        <v>350</v>
+      </c>
+      <c r="E22" s="13" t="n"/>
+      <c r="F22" s="13" t="n"/>
+      <c r="G22" s="13" t="n"/>
+      <c r="H22" s="13" t="n"/>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>30216123</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Marlo</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>Old Brown leather</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="n">
+        <v>350</v>
+      </c>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="13" t="n"/>
+      <c r="G23" s="13" t="n"/>
+      <c r="H23" s="13" t="n"/>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>30827772</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Marlo</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>Old White trim bridle side, leather top</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="n">
+        <v>350</v>
+      </c>
+      <c r="E24" s="13" t="n"/>
+      <c r="F24" s="13" t="n"/>
+      <c r="G24" s="13" t="n"/>
+      <c r="H24" s="13" t="n"/>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>30216387</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Marlo</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>Old White Trim Grey Leather</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="n">
+        <v>350</v>
+      </c>
+      <c r="E25" s="13" t="n"/>
+      <c r="F25" s="13" t="n"/>
+      <c r="G25" s="13" t="n"/>
+      <c r="H25" s="13" t="n"/>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>11207124</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Maverick</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Cowhide Front, Back</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="n">
+        <v>600</v>
+      </c>
+      <c r="E26" s="13" t="n"/>
+      <c r="F26" s="13" t="n"/>
+      <c r="G26" s="13" t="n"/>
+      <c r="H26" s="13" t="n"/>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>11207088</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Maverick</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>Floral</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="n">
+        <v>600</v>
+      </c>
+      <c r="E27" s="13" t="n"/>
+      <c r="F27" s="13" t="n"/>
+      <c r="G27" s="13" t="n"/>
+      <c r="H27" s="13" t="n"/>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Murphy</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>springbok</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E28" s="13" t="n"/>
+      <c r="F28" s="13" t="n"/>
+      <c r="G28" s="13" t="n"/>
+      <c r="H28" s="13" t="n"/>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Saddle</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Custom</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="E29" s="13" t="n"/>
+      <c r="F29" s="13" t="n"/>
+      <c r="G29" s="13" t="n"/>
+      <c r="H29" s="13" t="n"/>
+      <c r="I29" s="13" t="inlineStr">
+        <is>
+          <t>Custom line — not a photographed hide. Hidden on the site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>30400726</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Saddle</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Valentina Gold Rush</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="E30" s="13" t="n"/>
+      <c r="F30" s="13" t="n"/>
+      <c r="G30" s="13" t="n"/>
+      <c r="H30" s="13" t="n"/>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>SANTA-FE</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>3-piece sectional</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E31" s="13" t="n"/>
+      <c r="F31" s="13" t="n"/>
+      <c r="G31" s="13" t="n"/>
+      <c r="H31" s="13" t="n"/>
+      <c r="I31" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>11646333</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>Serena</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="n">
+        <v>600</v>
+      </c>
+      <c r="E32" s="13" t="n"/>
+      <c r="F32" s="13" t="n"/>
+      <c r="G32" s="13" t="n"/>
+      <c r="H32" s="13" t="n"/>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>30450724</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Smith</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>Tufted Valentina Tawny</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="n">
+        <v>150</v>
+      </c>
+      <c r="E33" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>Smith barstool Tufted Valentina Tawny</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="inlineStr">
+        <is>
+          <t>150 on master vs 200 at Sunset Sage</t>
+        </is>
+      </c>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>61633641</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Spring Buck</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>Springbuck</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E34" s="13" t="n"/>
+      <c r="F34" s="13" t="n"/>
+      <c r="G34" s="13" t="n"/>
+      <c r="H34" s="13" t="n"/>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>30101390</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Trophy</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Tufted Brown Leather</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="n">
+        <v>650</v>
+      </c>
+      <c r="E35" s="13" t="n"/>
+      <c r="F35" s="13" t="n"/>
+      <c r="G35" s="13" t="n"/>
+      <c r="H35" s="13" t="n"/>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>30102016</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Trophy</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>Tufted Dark Brown Leather</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="n">
+        <v>650</v>
+      </c>
+      <c r="E36" s="13" t="n"/>
+      <c r="F36" s="13" t="n"/>
+      <c r="G36" s="13" t="n"/>
+      <c r="H36" s="13" t="n"/>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>30103003</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Trophy</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>White Croc</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="n">
+        <v>650</v>
+      </c>
+      <c r="E37" s="13" t="n"/>
+      <c r="F37" s="13" t="n"/>
+      <c r="G37" s="13" t="n"/>
+      <c r="H37" s="13" t="n"/>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>30105382</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Trophy</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>Copper Embossed Leather</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="n">
+        <v>650</v>
+      </c>
+      <c r="E38" s="13" t="n"/>
+      <c r="F38" s="13" t="n"/>
+      <c r="G38" s="13" t="n"/>
+      <c r="H38" s="13" t="n"/>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>30110049</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Wilson</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Tufted Brown Back &amp; Seat</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="E39" s="13" t="n"/>
+      <c r="F39" s="13" t="n"/>
+      <c r="G39" s="13" t="n"/>
+      <c r="H39" s="13" t="n"/>
+      <c r="I39" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>NEW-SCOTT-BLACK</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>Scott</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="E40" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="F40" s="13" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>Scott Barstool black 25"</t>
+        </is>
+      </c>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>Not on master. 25" height. Assign a real SKU.</t>
+        </is>
+      </c>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>NEW-SCOTT-CAMEL</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>Scott</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>Camel</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="E41" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="F41" s="13" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="G41" s="13" t="inlineStr">
+        <is>
+          <t>Scott Barstool camel 25"</t>
+        </is>
+      </c>
+      <c r="H41" s="13" t="inlineStr">
+        <is>
+          <t>Not on master. 25" height. Assign a real SKU.</t>
+        </is>
+      </c>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>NEW-BROOKE-BAR-BLACK</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>Brooke</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="E42" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" s="13" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="G42" s="13" t="inlineStr">
+        <is>
+          <t>Brooke Black Barstool</t>
+        </is>
+      </c>
+      <c r="H42" s="13" t="inlineStr">
+        <is>
+          <t>Barstool, not dining. Assign a real SKU.</t>
+        </is>
+      </c>
+      <c r="I42" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>NEW-DAKOTA-TAUPE</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>Dakota</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>Taupe</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="E43" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="13" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="G43" s="13" t="inlineStr">
+        <is>
+          <t>Dakota dining chair Taupe</t>
+        </is>
+      </c>
+      <c r="H43" s="13" t="inlineStr">
+        <is>
+          <t>Not on master. Assign a real SKU.</t>
+        </is>
+      </c>
+      <c r="I43" s="13" t="inlineStr">
+        <is>
+          <t>No studio shot and not in the Sage inventory photos.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I43"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1198,7 +2601,7 @@
       </c>
       <c r="P5" s="8" t="inlineStr"/>
       <c r="Q5" s="8" t="inlineStr"/>
-      <c r="R5" s="8" t="inlineStr"/>
+      <c r="R5" s="11" t="inlineStr"/>
       <c r="S5" s="8" t="inlineStr"/>
       <c r="T5" s="8" t="inlineStr"/>
       <c r="U5" s="8" t="inlineStr"/>
@@ -1338,7 +2741,7 @@
       </c>
       <c r="P7" s="8" t="inlineStr"/>
       <c r="Q7" s="8" t="inlineStr"/>
-      <c r="R7" s="8" t="inlineStr"/>
+      <c r="R7" s="11" t="inlineStr"/>
       <c r="S7" s="8" t="inlineStr"/>
       <c r="T7" s="8" t="inlineStr"/>
       <c r="U7" s="8" t="inlineStr"/>
@@ -1408,7 +2811,7 @@
       </c>
       <c r="P8" s="8" t="inlineStr"/>
       <c r="Q8" s="8" t="inlineStr"/>
-      <c r="R8" s="8" t="inlineStr"/>
+      <c r="R8" s="11" t="inlineStr"/>
       <c r="S8" s="8" t="inlineStr"/>
       <c r="T8" s="8" t="inlineStr"/>
       <c r="U8" s="8" t="inlineStr"/>
@@ -1478,7 +2881,7 @@
       </c>
       <c r="P9" s="8" t="inlineStr"/>
       <c r="Q9" s="8" t="inlineStr"/>
-      <c r="R9" s="8" t="inlineStr"/>
+      <c r="R9" s="11" t="inlineStr"/>
       <c r="S9" s="8" t="inlineStr"/>
       <c r="T9" s="8" t="inlineStr"/>
       <c r="U9" s="8" t="inlineStr"/>
@@ -1548,7 +2951,7 @@
       </c>
       <c r="P10" s="8" t="inlineStr"/>
       <c r="Q10" s="8" t="inlineStr"/>
-      <c r="R10" s="8" t="inlineStr"/>
+      <c r="R10" s="11" t="inlineStr"/>
       <c r="S10" s="8" t="inlineStr"/>
       <c r="T10" s="8" t="inlineStr"/>
       <c r="U10" s="8" t="inlineStr"/>
@@ -1618,7 +3021,7 @@
       </c>
       <c r="P11" s="8" t="inlineStr"/>
       <c r="Q11" s="8" t="inlineStr"/>
-      <c r="R11" s="8" t="inlineStr"/>
+      <c r="R11" s="11" t="inlineStr"/>
       <c r="S11" s="8" t="inlineStr"/>
       <c r="T11" s="8" t="inlineStr"/>
       <c r="U11" s="8" t="inlineStr"/>
@@ -1688,7 +3091,7 @@
       </c>
       <c r="P12" s="8" t="inlineStr"/>
       <c r="Q12" s="8" t="inlineStr"/>
-      <c r="R12" s="8" t="inlineStr"/>
+      <c r="R12" s="11" t="inlineStr"/>
       <c r="S12" s="8" t="inlineStr"/>
       <c r="T12" s="8" t="inlineStr"/>
       <c r="U12" s="8" t="inlineStr"/>
@@ -2152,7 +3555,7 @@
       </c>
       <c r="P18" s="8" t="inlineStr"/>
       <c r="Q18" s="8" t="inlineStr"/>
-      <c r="R18" s="8" t="inlineStr"/>
+      <c r="R18" s="11" t="inlineStr"/>
       <c r="S18" s="8" t="inlineStr"/>
       <c r="T18" s="8" t="inlineStr"/>
       <c r="U18" s="8" t="inlineStr"/>
@@ -2718,7 +4121,7 @@
       <c r="Q26" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="R26" s="8" t="inlineStr"/>
+      <c r="R26" s="11" t="inlineStr"/>
       <c r="S26" s="8" t="inlineStr"/>
       <c r="T26" s="10" t="inlineStr">
         <is>
@@ -3970,7 +5373,7 @@
       </c>
       <c r="P43" s="8" t="inlineStr"/>
       <c r="Q43" s="8" t="inlineStr"/>
-      <c r="R43" s="8" t="inlineStr"/>
+      <c r="R43" s="11" t="inlineStr"/>
       <c r="S43" s="8" t="inlineStr"/>
       <c r="T43" s="8" t="inlineStr"/>
       <c r="U43" s="8" t="inlineStr"/>
@@ -4092,7 +5495,7 @@
       </c>
       <c r="P45" s="8" t="inlineStr"/>
       <c r="Q45" s="8" t="inlineStr"/>
-      <c r="R45" s="8" t="inlineStr"/>
+      <c r="R45" s="11" t="inlineStr"/>
       <c r="S45" s="8" t="inlineStr"/>
       <c r="T45" s="8" t="inlineStr"/>
       <c r="U45" s="8" t="inlineStr"/>
@@ -4154,7 +5557,7 @@
       </c>
       <c r="P46" s="8" t="inlineStr"/>
       <c r="Q46" s="8" t="inlineStr"/>
-      <c r="R46" s="8" t="inlineStr"/>
+      <c r="R46" s="11" t="inlineStr"/>
       <c r="S46" s="8" t="inlineStr"/>
       <c r="T46" s="8" t="inlineStr"/>
       <c r="U46" s="8" t="inlineStr"/>
@@ -4346,7 +5749,7 @@
       </c>
       <c r="P49" s="8" t="inlineStr"/>
       <c r="Q49" s="8" t="inlineStr"/>
-      <c r="R49" s="8" t="inlineStr"/>
+      <c r="R49" s="11" t="inlineStr"/>
       <c r="S49" s="8" t="inlineStr"/>
       <c r="T49" s="8" t="inlineStr"/>
       <c r="U49" s="8" t="inlineStr"/>
@@ -4878,7 +6281,7 @@
       </c>
       <c r="P56" s="8" t="inlineStr"/>
       <c r="Q56" s="8" t="inlineStr"/>
-      <c r="R56" s="8" t="inlineStr"/>
+      <c r="R56" s="11" t="inlineStr"/>
       <c r="S56" s="8" t="inlineStr"/>
       <c r="T56" s="8" t="inlineStr"/>
       <c r="U56" s="8" t="inlineStr"/>
@@ -5358,7 +6761,7 @@
       </c>
       <c r="P62" s="8" t="inlineStr"/>
       <c r="Q62" s="8" t="inlineStr"/>
-      <c r="R62" s="8" t="inlineStr"/>
+      <c r="R62" s="11" t="inlineStr"/>
       <c r="S62" s="8" t="inlineStr"/>
       <c r="T62" s="8" t="inlineStr"/>
       <c r="U62" s="8" t="inlineStr"/>
@@ -6626,7 +8029,7 @@
       </c>
       <c r="P78" s="8" t="inlineStr"/>
       <c r="Q78" s="8" t="inlineStr"/>
-      <c r="R78" s="8" t="inlineStr"/>
+      <c r="R78" s="11" t="inlineStr"/>
       <c r="S78" s="8" t="inlineStr"/>
       <c r="T78" s="8" t="inlineStr"/>
       <c r="U78" s="8" t="inlineStr"/>
@@ -6686,7 +8089,7 @@
       </c>
       <c r="P79" s="8" t="inlineStr"/>
       <c r="Q79" s="8" t="inlineStr"/>
-      <c r="R79" s="8" t="inlineStr"/>
+      <c r="R79" s="11" t="inlineStr"/>
       <c r="S79" s="8" t="inlineStr"/>
       <c r="T79" s="8" t="inlineStr"/>
       <c r="U79" s="8" t="inlineStr"/>
@@ -6746,7 +8149,7 @@
       </c>
       <c r="P80" s="8" t="inlineStr"/>
       <c r="Q80" s="8" t="inlineStr"/>
-      <c r="R80" s="8" t="inlineStr"/>
+      <c r="R80" s="11" t="inlineStr"/>
       <c r="S80" s="8" t="inlineStr"/>
       <c r="T80" s="8" t="inlineStr"/>
       <c r="U80" s="8" t="inlineStr"/>
@@ -6940,7 +8343,7 @@
       </c>
       <c r="P83" s="8" t="inlineStr"/>
       <c r="Q83" s="8" t="inlineStr"/>
-      <c r="R83" s="8" t="inlineStr"/>
+      <c r="R83" s="11" t="inlineStr"/>
       <c r="S83" s="8" t="inlineStr"/>
       <c r="T83" s="8" t="inlineStr"/>
       <c r="U83" s="8" t="inlineStr"/>
@@ -7610,7 +9013,7 @@
       </c>
       <c r="P92" s="8" t="inlineStr"/>
       <c r="Q92" s="8" t="inlineStr"/>
-      <c r="R92" s="8" t="inlineStr"/>
+      <c r="R92" s="11" t="inlineStr"/>
       <c r="S92" s="8" t="inlineStr"/>
       <c r="T92" s="8" t="inlineStr"/>
       <c r="U92" s="8" t="inlineStr"/>
@@ -7676,7 +9079,7 @@
       </c>
       <c r="P93" s="8" t="inlineStr"/>
       <c r="Q93" s="8" t="inlineStr"/>
-      <c r="R93" s="8" t="inlineStr"/>
+      <c r="R93" s="11" t="inlineStr"/>
       <c r="S93" s="8" t="inlineStr"/>
       <c r="T93" s="8" t="inlineStr"/>
       <c r="U93" s="8" t="inlineStr"/>
@@ -7742,7 +9145,7 @@
       </c>
       <c r="P94" s="8" t="inlineStr"/>
       <c r="Q94" s="8" t="inlineStr"/>
-      <c r="R94" s="8" t="inlineStr"/>
+      <c r="R94" s="11" t="inlineStr"/>
       <c r="S94" s="8" t="inlineStr"/>
       <c r="T94" s="8" t="inlineStr"/>
       <c r="U94" s="8" t="inlineStr"/>
@@ -7874,7 +9277,7 @@
       </c>
       <c r="P96" s="8" t="inlineStr"/>
       <c r="Q96" s="8" t="inlineStr"/>
-      <c r="R96" s="8" t="inlineStr"/>
+      <c r="R96" s="11" t="inlineStr"/>
       <c r="S96" s="8" t="inlineStr"/>
       <c r="T96" s="8" t="inlineStr"/>
       <c r="U96" s="8" t="inlineStr"/>
@@ -7940,7 +9343,7 @@
       </c>
       <c r="P97" s="8" t="inlineStr"/>
       <c r="Q97" s="8" t="inlineStr"/>
-      <c r="R97" s="8" t="inlineStr"/>
+      <c r="R97" s="11" t="inlineStr"/>
       <c r="S97" s="8" t="inlineStr"/>
       <c r="T97" s="8" t="inlineStr"/>
       <c r="U97" s="8" t="inlineStr"/>
@@ -8080,7 +9483,7 @@
       </c>
       <c r="P99" s="8" t="inlineStr"/>
       <c r="Q99" s="8" t="inlineStr"/>
-      <c r="R99" s="8" t="inlineStr"/>
+      <c r="R99" s="11" t="inlineStr"/>
       <c r="S99" s="8" t="inlineStr"/>
       <c r="T99" s="8" t="inlineStr"/>
       <c r="U99" s="8" t="inlineStr"/>
@@ -8310,7 +9713,7 @@
       </c>
       <c r="P102" s="8" t="inlineStr"/>
       <c r="Q102" s="8" t="inlineStr"/>
-      <c r="R102" s="8" t="inlineStr"/>
+      <c r="R102" s="11" t="inlineStr"/>
       <c r="S102" s="8" t="inlineStr"/>
       <c r="T102" s="8" t="inlineStr"/>
       <c r="U102" s="8" t="inlineStr"/>
@@ -8372,7 +9775,7 @@
       </c>
       <c r="P103" s="8" t="inlineStr"/>
       <c r="Q103" s="8" t="inlineStr"/>
-      <c r="R103" s="8" t="inlineStr"/>
+      <c r="R103" s="11" t="inlineStr"/>
       <c r="S103" s="8" t="inlineStr"/>
       <c r="T103" s="8" t="inlineStr"/>
       <c r="U103" s="8" t="inlineStr"/>
@@ -10838,7 +12241,7 @@
       </c>
       <c r="P134" s="8" t="inlineStr"/>
       <c r="Q134" s="8" t="inlineStr"/>
-      <c r="R134" s="8" t="inlineStr"/>
+      <c r="R134" s="11" t="inlineStr"/>
       <c r="S134" s="8" t="inlineStr"/>
       <c r="T134" s="8" t="inlineStr"/>
       <c r="U134" s="8" t="inlineStr"/>
@@ -10902,7 +12305,7 @@
       </c>
       <c r="P135" s="8" t="inlineStr"/>
       <c r="Q135" s="8" t="inlineStr"/>
-      <c r="R135" s="8" t="inlineStr"/>
+      <c r="R135" s="11" t="inlineStr"/>
       <c r="S135" s="8" t="inlineStr"/>
       <c r="T135" s="8" t="inlineStr"/>
       <c r="U135" s="8" t="inlineStr"/>
@@ -11062,7 +12465,7 @@
       </c>
       <c r="P137" s="8" t="inlineStr"/>
       <c r="Q137" s="8" t="inlineStr"/>
-      <c r="R137" s="8" t="inlineStr"/>
+      <c r="R137" s="11" t="inlineStr"/>
       <c r="S137" s="8" t="inlineStr"/>
       <c r="T137" s="8" t="inlineStr"/>
       <c r="U137" s="8" t="inlineStr"/>
@@ -11408,7 +12811,7 @@
       <c r="Q142" s="8" t="n">
         <v>200</v>
       </c>
-      <c r="R142" s="8" t="inlineStr"/>
+      <c r="R142" s="11" t="inlineStr"/>
       <c r="S142" s="8" t="inlineStr"/>
       <c r="T142" s="9" t="inlineStr">
         <is>
@@ -11482,7 +12885,7 @@
       </c>
       <c r="P143" s="8" t="inlineStr"/>
       <c r="Q143" s="8" t="inlineStr"/>
-      <c r="R143" s="8" t="inlineStr"/>
+      <c r="R143" s="11" t="inlineStr"/>
       <c r="S143" s="8" t="inlineStr"/>
       <c r="T143" s="8" t="inlineStr"/>
       <c r="U143" s="8" t="inlineStr"/>
@@ -11898,7 +13301,7 @@
       </c>
       <c r="P149" s="8" t="inlineStr"/>
       <c r="Q149" s="8" t="inlineStr"/>
-      <c r="R149" s="8" t="inlineStr"/>
+      <c r="R149" s="11" t="inlineStr"/>
       <c r="S149" s="8" t="inlineStr"/>
       <c r="T149" s="8" t="inlineStr"/>
       <c r="U149" s="8" t="inlineStr"/>
@@ -12380,7 +13783,7 @@
       </c>
       <c r="P156" s="8" t="inlineStr"/>
       <c r="Q156" s="8" t="inlineStr"/>
-      <c r="R156" s="8" t="inlineStr"/>
+      <c r="R156" s="11" t="inlineStr"/>
       <c r="S156" s="8" t="inlineStr"/>
       <c r="T156" s="8" t="inlineStr"/>
       <c r="U156" s="8" t="inlineStr"/>
@@ -13296,7 +14699,7 @@
       </c>
       <c r="P168" s="8" t="inlineStr"/>
       <c r="Q168" s="8" t="inlineStr"/>
-      <c r="R168" s="8" t="inlineStr"/>
+      <c r="R168" s="11" t="inlineStr"/>
       <c r="S168" s="8" t="inlineStr"/>
       <c r="T168" s="8" t="inlineStr"/>
       <c r="U168" s="8" t="inlineStr"/>
@@ -13428,7 +14831,7 @@
       </c>
       <c r="P170" s="8" t="inlineStr"/>
       <c r="Q170" s="8" t="inlineStr"/>
-      <c r="R170" s="8" t="inlineStr"/>
+      <c r="R170" s="11" t="inlineStr"/>
       <c r="S170" s="8" t="inlineStr"/>
       <c r="T170" s="8" t="inlineStr"/>
       <c r="U170" s="8" t="inlineStr"/>
@@ -14272,7 +15675,7 @@
       </c>
       <c r="P181" s="8" t="inlineStr"/>
       <c r="Q181" s="8" t="inlineStr"/>
-      <c r="R181" s="8" t="inlineStr"/>
+      <c r="R181" s="11" t="inlineStr"/>
       <c r="S181" s="8" t="inlineStr"/>
       <c r="T181" s="8" t="inlineStr"/>
       <c r="U181" s="8" t="inlineStr"/>
@@ -14524,7 +15927,7 @@
       <c r="Q185" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="R185" s="8" t="inlineStr"/>
+      <c r="R185" s="11" t="inlineStr"/>
       <c r="S185" s="8" t="inlineStr"/>
       <c r="T185" s="12" t="inlineStr">
         <is>
@@ -14660,7 +16063,7 @@
       <c r="Q187" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="R187" s="8" t="inlineStr"/>
+      <c r="R187" s="11" t="inlineStr"/>
       <c r="S187" s="8" t="inlineStr"/>
       <c r="T187" s="12" t="inlineStr">
         <is>
@@ -15212,7 +16615,7 @@
       <c r="Q195" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="R195" s="8" t="inlineStr"/>
+      <c r="R195" s="11" t="inlineStr"/>
       <c r="S195" s="8" t="inlineStr"/>
       <c r="T195" s="12" t="inlineStr">
         <is>
@@ -15554,7 +16957,7 @@
       <c r="Q200" s="8" t="n">
         <v>500</v>
       </c>
-      <c r="R200" s="8" t="inlineStr"/>
+      <c r="R200" s="11" t="inlineStr"/>
       <c r="S200" s="8" t="inlineStr"/>
       <c r="T200" s="12" t="inlineStr">
         <is>
@@ -15578,7 +16981,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16051,7 +17454,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16702,7 +18105,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>